<commit_message>
comment code of email send of audit application received, added code for excel report download for manager, added markdown in auditor audit list page
</commit_message>
<xml_diff>
--- a/client_report/service/tests/snapshots/get_xlsx_report_for_clientuser_1.xlsx
+++ b/client_report/service/tests/snapshots/get_xlsx_report_for_clientuser_1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="59">
   <si>
     <t>Audit Report</t>
   </si>
@@ -115,18 +115,12 @@
     <t>Was there place to keep helmet and bags?</t>
   </si>
   <si>
-    <t>Auditor Comment</t>
+    <t>Section Summary</t>
   </si>
   <si>
     <t>entrance was visible and welcoming</t>
   </si>
   <si>
-    <t>PM Comment</t>
-  </si>
-  <si>
-    <t>no security guard</t>
-  </si>
-  <si>
     <t>Did the staff greet you upon arrival?</t>
   </si>
   <si>
@@ -145,9 +139,6 @@
     <t>my need was not asked</t>
   </si>
   <si>
-    <t>not so good staff</t>
-  </si>
-  <si>
     <t>Did the staff member address you by saying 'Sir' or 'Madam'?</t>
   </si>
   <si>
@@ -166,9 +157,6 @@
     <t>staff was not looking very interested</t>
   </si>
   <si>
-    <t>staff not interested</t>
-  </si>
-  <si>
     <t>Did the staff ask for your budget before starting to show products?</t>
   </si>
   <si>
@@ -187,9 +175,6 @@
     <t>selling skills were quite poor</t>
   </si>
   <si>
-    <t>no selling skills</t>
-  </si>
-  <si>
     <t>Was the outlet neat and clean?</t>
   </si>
   <si>
@@ -206,9 +191,6 @@
   </si>
   <si>
     <t>outlet was quite clean and presentable</t>
-  </si>
-  <si>
-    <t>good showroom</t>
   </si>
 </sst>
 </file>
@@ -240,7 +222,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -277,12 +259,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFBF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -311,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -326,9 +302,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -625,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:E57"/>
+  <dimension ref="A2:E52"/>
   <sheetFormatPr defaultRowHeight="20" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -873,41 +846,45 @@
       <c r="E20" s="5"/>
     </row>
     <row r="21" spans="1:5" ht="20" customHeight="1">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6" t="s">
+      <c r="A21" s="3">
+        <v>2</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="20" customHeight="1">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-    </row>
-    <row r="22" spans="1:5" ht="20" customHeight="1">
-      <c r="A22" s="3">
-        <v>2</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3">
-        <v>3</v>
-      </c>
-      <c r="E22" s="3">
-        <v>5</v>
+      <c r="C22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="20" customHeight="1">
       <c r="A23" s="4"/>
       <c r="B23" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D23" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="4">
         <v>1</v>
@@ -916,13 +893,13 @@
     <row r="24" spans="1:5" ht="20" customHeight="1">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D24" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="2">
         <v>1</v>
@@ -931,7 +908,7 @@
     <row r="25" spans="1:5" ht="20" customHeight="1">
       <c r="A25" s="4"/>
       <c r="B25" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>27</v>
@@ -946,74 +923,78 @@
     <row r="26" spans="1:5" ht="20" customHeight="1">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" s="2">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="20" customHeight="1">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D26" s="2">
-        <v>1</v>
-      </c>
-      <c r="E26" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="20" customHeight="1">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4" t="s">
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+    </row>
+    <row r="29" spans="1:5" ht="20" customHeight="1">
+      <c r="A29" s="3">
+        <v>3</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3">
+        <v>4</v>
+      </c>
+      <c r="E29" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="20" customHeight="1">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D27" s="4">
-        <v>0</v>
-      </c>
-      <c r="E27" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="20" customHeight="1">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C29" s="5" t="s">
+      <c r="C30" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" s="4">
+        <v>1</v>
+      </c>
+      <c r="E30" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="20" customHeight="1">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-    </row>
-    <row r="30" spans="1:5" ht="20" customHeight="1">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-    </row>
-    <row r="31" spans="1:5" ht="20" customHeight="1">
-      <c r="A31" s="3">
-        <v>3</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3">
-        <v>4</v>
-      </c>
-      <c r="E31" s="3">
-        <v>5</v>
+      <c r="C31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="2">
+        <v>1</v>
+      </c>
+      <c r="E31" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="20" customHeight="1">
       <c r="A32" s="4"/>
       <c r="B32" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>27</v>
@@ -1028,7 +1009,7 @@
     <row r="33" spans="1:5" ht="20" customHeight="1">
       <c r="A33" s="2"/>
       <c r="B33" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>27</v>
@@ -1043,95 +1024,99 @@
     <row r="34" spans="1:5" ht="20" customHeight="1">
       <c r="A34" s="4"/>
       <c r="B34" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D34" s="4">
+        <v>0</v>
+      </c>
+      <c r="E34" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="20" customHeight="1">
+      <c r="A36" s="5"/>
+      <c r="B36" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D34" s="4">
-        <v>1</v>
-      </c>
-      <c r="E34" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="20" customHeight="1">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2" t="s">
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+    </row>
+    <row r="37" spans="1:5" ht="20" customHeight="1">
+      <c r="A37" s="3">
+        <v>4</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3">
+        <v>2</v>
+      </c>
+      <c r="E37" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="20" customHeight="1">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D35" s="2">
-        <v>1</v>
-      </c>
-      <c r="E35" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="20" customHeight="1">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4" t="s">
+      <c r="C38" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D38" s="2">
+        <v>0</v>
+      </c>
+      <c r="E38" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="20" customHeight="1">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C39" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D36" s="4">
+      <c r="D39" s="4">
         <v>0</v>
       </c>
-      <c r="E36" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="20" customHeight="1">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C38" s="5" t="s">
+      <c r="E39" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="20" customHeight="1">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-    </row>
-    <row r="39" spans="1:5" ht="20" customHeight="1">
-      <c r="A39" s="6"/>
-      <c r="B39" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-    </row>
-    <row r="40" spans="1:5" ht="20" customHeight="1">
-      <c r="A40" s="3">
-        <v>4</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3">
-        <v>2</v>
-      </c>
-      <c r="E40" s="3">
-        <v>5</v>
+      <c r="C40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D40" s="2">
+        <v>1</v>
+      </c>
+      <c r="E40" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="20" customHeight="1">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D41" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" s="4">
         <v>1</v>
@@ -1140,7 +1125,7 @@
     <row r="42" spans="1:5" ht="20" customHeight="1">
       <c r="A42" s="2"/>
       <c r="B42" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>31</v>
@@ -1152,184 +1137,117 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="20" customHeight="1">
-      <c r="A43" s="4"/>
-      <c r="B43" s="4" t="s">
+    <row r="44" spans="1:5" ht="20" customHeight="1">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+    </row>
+    <row r="45" spans="1:5" ht="20" customHeight="1">
+      <c r="A45" s="3">
+        <v>5</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3">
+        <v>5</v>
+      </c>
+      <c r="E45" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="20" customHeight="1">
+      <c r="A46" s="4"/>
+      <c r="B46" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D43" s="4">
-        <v>1</v>
-      </c>
-      <c r="E43" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="20" customHeight="1">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2" t="s">
+      <c r="C46" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D46" s="4">
+        <v>1</v>
+      </c>
+      <c r="E46" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="20" customHeight="1">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D44" s="2">
-        <v>1</v>
-      </c>
-      <c r="E44" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="20" customHeight="1">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4" t="s">
+      <c r="C47" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D47" s="2">
+        <v>1</v>
+      </c>
+      <c r="E47" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="20" customHeight="1">
+      <c r="A48" s="4"/>
+      <c r="B48" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C45" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D45" s="4">
-        <v>0</v>
-      </c>
-      <c r="E45" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="20" customHeight="1">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C47" s="5" t="s">
+      <c r="C48" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D48" s="4">
+        <v>1</v>
+      </c>
+      <c r="E48" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="20" customHeight="1">
+      <c r="A49" s="2"/>
+      <c r="B49" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
-    </row>
-    <row r="48" spans="1:5" ht="20" customHeight="1">
-      <c r="A48" s="6"/>
-      <c r="B48" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-    </row>
-    <row r="49" spans="1:5" ht="20" customHeight="1">
-      <c r="A49" s="3">
-        <v>5</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3">
-        <v>5</v>
-      </c>
-      <c r="E49" s="3">
-        <v>5</v>
+      <c r="C49" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D49" s="2">
+        <v>1</v>
+      </c>
+      <c r="E49" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="20" customHeight="1">
       <c r="A50" s="4"/>
       <c r="B50" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D50" s="4">
+        <v>1</v>
+      </c>
+      <c r="E50" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="20" customHeight="1">
+      <c r="A52" s="5"/>
+      <c r="B52" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C52" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C50" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D50" s="4">
-        <v>1</v>
-      </c>
-      <c r="E50" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="20" customHeight="1">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D51" s="2">
-        <v>1</v>
-      </c>
-      <c r="E51" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="20" customHeight="1">
-      <c r="A52" s="4"/>
-      <c r="B52" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D52" s="4">
-        <v>1</v>
-      </c>
-      <c r="E52" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="20" customHeight="1">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D53" s="2">
-        <v>1</v>
-      </c>
-      <c r="E53" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="20" customHeight="1">
-      <c r="A54" s="4"/>
-      <c r="B54" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D54" s="4">
-        <v>1</v>
-      </c>
-      <c r="E54" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="20" customHeight="1">
-      <c r="A56" s="5"/>
-      <c r="B56" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
-    </row>
-    <row r="57" spans="1:5" ht="20" customHeight="1">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="D57" s="6"/>
-      <c r="E57" s="6"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>